<commit_message>
fix(central): the template's topic column is rebuilt from one source of truth
It used to APPEND to whatever the source workbook had, which is precisely how the
served template and the live tag set drifted apart -- 24 department names went in
that way and the taxonomy has now dropped them. The column is rebuilt from
DEFAULT_QUESTION_TAGS, so the file an admin downloads and the list the importer
validates against cannot disagree.

Still edited in place, never regenerated: styles, theme, the other two sheets and
the Context drop-down all survive byte-identical.

Date: 2026-08-26 20:46 UTC
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scrutinise-web/public/central-question-upload-template.xlsx
+++ b/scrutinise-web/public/central-question-upload-template.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="89">
   <si>
     <t>Scrutinise Central — bulk question upload template</t>
   </si>
@@ -246,76 +246,49 @@
     <t>Our local branch is a mature political movement fully realigned from the Uniparty</t>
   </si>
   <si>
-    <t>Attorney General’s Office</t>
-  </si>
-  <si>
-    <t>Cabinet Office</t>
-  </si>
-  <si>
-    <t>Department for Business and Trade</t>
-  </si>
-  <si>
-    <t>Department for Culture, Media and Sport</t>
-  </si>
-  <si>
-    <t>Department for Education</t>
-  </si>
-  <si>
-    <t>Department for Energy Security and Net Zero</t>
-  </si>
-  <si>
-    <t>Department for Environment, Food and Rural Affairs</t>
-  </si>
-  <si>
-    <t>Department for Science, Innovation and Technology</t>
-  </si>
-  <si>
-    <t>Department for Transport</t>
-  </si>
-  <si>
-    <t>Department for Work and Pensions</t>
-  </si>
-  <si>
-    <t>Department of Health and Social Care</t>
-  </si>
-  <si>
-    <t>Foreign, Commonwealth and Development Office</t>
-  </si>
-  <si>
-    <t>HM Treasury</t>
-  </si>
-  <si>
-    <t>Home Office</t>
-  </si>
-  <si>
-    <t>Ministry of Defence</t>
-  </si>
-  <si>
-    <t>Ministry of Housing, Communities and Local Government</t>
-  </si>
-  <si>
-    <t>Ministry of Justice</t>
-  </si>
-  <si>
-    <t>Northern Ireland Office</t>
-  </si>
-  <si>
-    <t>Office of the Advocate General for Scotland</t>
-  </si>
-  <si>
-    <t>Office of the Leader of the House of Commons</t>
-  </si>
-  <si>
-    <t>Office of the Leader of the House of Lords</t>
-  </si>
-  <si>
-    <t>Scotland Office</t>
-  </si>
-  <si>
-    <t>UK Export Finance</t>
-  </si>
-  <si>
-    <t>Wales Office</t>
+    <t>Immigration &amp; asylum</t>
+  </si>
+  <si>
+    <t>Crime, justice &amp; policing</t>
+  </si>
+  <si>
+    <t>Health &amp; care</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>Transport &amp; roads</t>
+  </si>
+  <si>
+    <t>Energy &amp; net zero</t>
+  </si>
+  <si>
+    <t>Environment, farming &amp; rural</t>
+  </si>
+  <si>
+    <t>Economy &amp; tax</t>
+  </si>
+  <si>
+    <t>Welfare &amp; pensions</t>
+  </si>
+  <si>
+    <t>Business &amp; jobs</t>
+  </si>
+  <si>
+    <t>Culture, media &amp; sport</t>
+  </si>
+  <si>
+    <t>Science, technology &amp; digital</t>
+  </si>
+  <si>
+    <t>Defence &amp; foreign affairs</t>
+  </si>
+  <si>
+    <t>Constitution, devolution &amp; elections</t>
+  </si>
+  <si>
+    <t>Social &amp; moral issues</t>
   </si>
 </sst>
 </file>
@@ -2825,7 +2798,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="26" customWidth="1"/>
@@ -2851,7 +2824,7 @@
         <v>55</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -2862,7 +2835,7 @@
         <v>55</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -2873,7 +2846,7 @@
         <v>55</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -2884,7 +2857,7 @@
         <v>55</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -2895,7 +2868,7 @@
         <v>55</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -2906,7 +2879,7 @@
         <v>64</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -2917,7 +2890,7 @@
         <v>64</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -2928,146 +2901,81 @@
         <v>64</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="C10" s="9" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="C11" s="9" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="C12" s="9" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="C13" s="9" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="C14" s="9" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="C15" s="9" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="C16" s="9" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="C17" s="9" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="C18" s="9" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="C19" s="9" t="s">
-        <v>80</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="C20" s="9" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="C21" s="9" t="s">
-        <v>82</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="C22" s="9" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="C23" s="9" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="C24" s="9" t="s">
-        <v>85</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:3">
-      <c r="C25" s="9" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="C26" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="C27" s="9" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="C28" s="9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3">
-      <c r="C29" s="9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="C30" s="9" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="C31" s="9" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="C32" s="9" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3">
-      <c r="C33" s="9" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="C34" s="9" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="C35" s="9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="C36" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3">
-      <c r="A38" s="10" t="s">
+      <c r="A25" s="10" t="s">
         <v>71</v>
       </c>
     </row>

</xml_diff>